<commit_message>
feat: add Selenium test suite for AI Quiz Generator and Chatbot features with supporting Excel data file
</commit_message>
<xml_diff>
--- a/data/TC_AIFeatures.xlsx
+++ b/data/TC_AIFeatures.xlsx
@@ -537,7 +537,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:L15"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="36" customWidth="1" min="2" max="2"/>
@@ -740,7 +740,7 @@
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
-          <t>Login failed</t>
+          <t>Could not reach Questions step (URL: https://datn-quizapp.web.app/creator/new)</t>
         </is>
       </c>
       <c r="I6" s="3" t="inlineStr">
@@ -760,7 +760,7 @@
       </c>
       <c r="L6" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"> | Run: 2026-04-18 12:25</t>
+          <t xml:space="preserve"> | Run: 2026-04-18 12:25 | Run: 2026-04-20 09:51 | Run: 2026-04-20 10:03</t>
         </is>
       </c>
     </row>
@@ -822,7 +822,7 @@
       </c>
       <c r="L7" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve"> | Run: 2026-04-18 12:25</t>
+          <t xml:space="preserve"> | Run: 2026-04-18 12:25 | Run: 2026-04-20 10:04</t>
         </is>
       </c>
     </row>
@@ -864,7 +864,7 @@
       </c>
       <c r="H8" s="3" t="inlineStr">
         <is>
-          <t>Login failed</t>
+          <t>Could not reach Questions step (URL: https://datn-quizapp.web.app/creator/new)</t>
         </is>
       </c>
       <c r="I8" s="3" t="inlineStr">
@@ -884,7 +884,7 @@
       </c>
       <c r="L8" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"> | Run: 2026-04-18 12:25</t>
+          <t xml:space="preserve"> | Run: 2026-04-18 12:25 | Run: 2026-04-20 10:05</t>
         </is>
       </c>
     </row>
@@ -926,7 +926,7 @@
       </c>
       <c r="H9" s="5" t="inlineStr">
         <is>
-          <t>Login failed</t>
+          <t>Could not reach Questions step (URL: https://datn-quizapp.web.app/creator/new)</t>
         </is>
       </c>
       <c r="I9" s="5" t="inlineStr">
@@ -946,7 +946,7 @@
       </c>
       <c r="L9" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve"> | Run: 2026-04-18 12:25</t>
+          <t xml:space="preserve"> | Run: 2026-04-18 12:25 | Run: 2026-04-20 10:07</t>
         </is>
       </c>
     </row>
@@ -988,7 +988,7 @@
       </c>
       <c r="H10" s="3" t="inlineStr">
         <is>
-          <t>Login failed</t>
+          <t>Could not reach Questions step (URL: https://datn-quizapp.web.app/creator/new)</t>
         </is>
       </c>
       <c r="I10" s="3" t="inlineStr">
@@ -1008,7 +1008,7 @@
       </c>
       <c r="L10" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"> | Run: 2026-04-18 12:26</t>
+          <t xml:space="preserve"> | Run: 2026-04-18 12:26 | Run: 2026-04-20 10:09</t>
         </is>
       </c>
     </row>
@@ -1050,7 +1050,7 @@
       </c>
       <c r="H11" s="5" t="inlineStr">
         <is>
-          <t>Login failed</t>
+          <t>Could not reach Questions step (URL: https://datn-quizapp.web.app/creator/new)</t>
         </is>
       </c>
       <c r="I11" s="5" t="inlineStr">
@@ -1070,7 +1070,7 @@
       </c>
       <c r="L11" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve"> | Run: 2026-04-18 12:26</t>
+          <t xml:space="preserve"> | Run: 2026-04-18 12:26 | Run: 2026-04-20 10:11</t>
         </is>
       </c>
     </row>
@@ -1132,7 +1132,7 @@
       </c>
       <c r="L12" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"> | Run: 2026-04-18 12:26</t>
+          <t xml:space="preserve"> | Run: 2026-04-18 12:26 | Run: 2026-04-20 10:12</t>
         </is>
       </c>
     </row>
@@ -1174,12 +1174,12 @@
       </c>
       <c r="H13" s="5" t="inlineStr">
         <is>
-          <t>User login failed</t>
+          <t>USER navigated to /creator/new → landed at: https://datn-quizapp.web.app/creator/new</t>
         </is>
       </c>
       <c r="I13" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>No data saved (USER role blocked from creator route); Firestore role='creator'</t>
         </is>
       </c>
       <c r="J13" s="5" t="inlineStr">
@@ -1194,7 +1194,7 @@
       </c>
       <c r="L13" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve"> | Run: 2026-04-18 12:26</t>
+          <t xml:space="preserve"> | Run: 2026-04-18 12:26 | Run: 2026-04-20 10:13</t>
         </is>
       </c>
     </row>
@@ -1236,7 +1236,7 @@
       </c>
       <c r="H14" s="3" t="inlineStr">
         <is>
-          <t>Login failed</t>
+          <t>Could not reach Questions step (URL: https://datn-quizapp.web.app/creator/new)</t>
         </is>
       </c>
       <c r="I14" s="3" t="inlineStr">
@@ -1256,7 +1256,7 @@
       </c>
       <c r="L14" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"> | Run: 2026-04-18 12:26</t>
+          <t xml:space="preserve"> | Run: 2026-04-18 12:26 | Run: 2026-04-20 10:15</t>
         </is>
       </c>
     </row>
@@ -1298,7 +1298,7 @@
       </c>
       <c r="H15" s="5" t="inlineStr">
         <is>
-          <t>Login failed</t>
+          <t>Could not reach Questions step (URL: https://datn-quizapp.web.app/creator/new)</t>
         </is>
       </c>
       <c r="I15" s="5" t="inlineStr">
@@ -1318,7 +1318,7 @@
       </c>
       <c r="L15" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve"> | Run: 2026-04-18 12:27</t>
+          <t xml:space="preserve"> | Run: 2026-04-18 12:27 | Run: 2026-04-20 10:16</t>
         </is>
       </c>
     </row>
@@ -1340,7 +1340,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:K17"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="36" customWidth="1" min="2" max="2"/>
@@ -1537,13 +1537,21 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="I6" s="3" t="n"/>
+      <c r="I6" s="3" t="inlineStr">
+        <is>
+          <t>Response: ''</t>
+        </is>
+      </c>
       <c r="J6" s="4" t="inlineStr">
         <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="K6" s="3" t="n"/>
+          <t>No DB state created</t>
+        </is>
+      </c>
+      <c r="K6" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> | Run: 2026-04-20 10:22</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
@@ -1586,13 +1594,21 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="I7" s="5" t="n"/>
+      <c r="I7" s="5" t="inlineStr">
+        <is>
+          <t>Send button disabled when input empty: True</t>
+        </is>
+      </c>
       <c r="J7" s="4" t="inlineStr">
         <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="K7" s="5" t="n"/>
+          <t>No API call triggered</t>
+        </is>
+      </c>
+      <c r="K7" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> | Run: 2026-04-20 10:24</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="25.5" customHeight="1">
       <c r="A8" s="3" t="inlineStr">
@@ -1635,13 +1651,21 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="I8" s="3" t="n"/>
+      <c r="I8" s="3" t="inlineStr">
+        <is>
+          <t>Response (0 chars): ''</t>
+        </is>
+      </c>
       <c r="J8" s="4" t="inlineStr">
         <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="K8" s="3" t="n"/>
+          <t>Citations found: False</t>
+        </is>
+      </c>
+      <c r="K8" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> | Run: 2026-04-20 10:26</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="25.5" customHeight="1">
       <c r="A9" s="5" t="inlineStr">
@@ -1684,13 +1708,21 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="I9" s="5" t="n"/>
+      <c r="I9" s="5" t="inlineStr">
+        <is>
+          <t>Response to 'a': ''; Known '0' bug: False</t>
+        </is>
+      </c>
       <c r="J9" s="4" t="inlineStr">
         <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="K9" s="5" t="n"/>
+          <t>No crash; no hallucination</t>
+        </is>
+      </c>
+      <c r="K9" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> | Run: 2026-04-20 10:28</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="409.5" customHeight="1">
       <c r="A10" s="3" t="inlineStr">
@@ -1782,13 +1814,21 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="I11" s="5" t="n"/>
+      <c r="I11" s="5" t="inlineStr">
+        <is>
+          <t>Response (0 chars): ''</t>
+        </is>
+      </c>
       <c r="J11" s="4" t="inlineStr">
         <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="K11" s="5" t="n"/>
+          <t>Citations found: False</t>
+        </is>
+      </c>
+      <c r="K11" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> | Run: 2026-04-20 10:31</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
@@ -1831,13 +1871,21 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="I12" s="3" t="n"/>
+      <c r="I12" s="3" t="inlineStr">
+        <is>
+          <t>Response: ''</t>
+        </is>
+      </c>
       <c r="J12" s="4" t="inlineStr">
         <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="K12" s="3" t="n"/>
+          <t>No session state written</t>
+        </is>
+      </c>
+      <c r="K12" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> | Run: 2026-04-20 10:34</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="25.5" customHeight="1">
       <c r="A13" s="5" t="inlineStr">
@@ -1929,13 +1977,21 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="I14" s="3" t="n"/>
+      <c r="I14" s="3" t="inlineStr">
+        <is>
+          <t>Response to 'lo den la gi': ''</t>
+        </is>
+      </c>
       <c r="J14" s="4" t="inlineStr">
         <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="K14" s="3" t="n"/>
+          <t>Diacritic-insensitive retrieval successful: False</t>
+        </is>
+      </c>
+      <c r="K14" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> | Run: 2026-04-20 10:38</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="25.5" customHeight="1">
       <c r="A15" s="5" t="inlineStr">
@@ -1978,13 +2034,21 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="I15" s="5" t="n"/>
+      <c r="I15" s="5" t="inlineStr">
+        <is>
+          <t>Phase indicators seen → Retrieve: False, Generate: False, Generic only: True</t>
+        </is>
+      </c>
       <c r="J15" s="4" t="inlineStr">
         <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="K15" s="5" t="n"/>
+          <t>N/A – UI-only streaming indicator check</t>
+        </is>
+      </c>
+      <c r="K15" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> | Run: 2026-04-20 10:39</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="25.5" customHeight="1">
       <c r="A16" s="3" t="inlineStr">
@@ -2027,13 +2091,21 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="I16" s="3" t="n"/>
+      <c r="I16" s="3" t="inlineStr">
+        <is>
+          <t>Raw Markdown visible: False; Rendered HTML elements present: False; Snippet: ''</t>
+        </is>
+      </c>
       <c r="J16" s="4" t="inlineStr">
         <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="K16" s="3" t="n"/>
+          <t>N/A – UI-only rendering check</t>
+        </is>
+      </c>
+      <c r="K16" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> | Run: 2026-04-20 10:41</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
@@ -2076,13 +2148,21 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="I17" s="5" t="n"/>
+      <c r="I17" s="5" t="inlineStr">
+        <is>
+          <t>Response appeared in 642.9s (threshold: 10s)</t>
+        </is>
+      </c>
       <c r="J17" s="4" t="inlineStr">
         <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="K17" s="5" t="n"/>
+          <t>Performance within threshold</t>
+        </is>
+      </c>
+      <c r="K17" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> | Run: 2026-04-20 10:53</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="4">

</xml_diff>

<commit_message>
feat: add Selenium test suite for AI Quiz Generator and Chatbot features
</commit_message>
<xml_diff>
--- a/data/TC_AIFeatures.xlsx
+++ b/data/TC_AIFeatures.xlsx
@@ -740,7 +740,7 @@
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
-          <t>Could not reach Questions step (URL: https://datn-quizapp.web.app/creator/new)</t>
+          <t>Preview shows 5 question card(s). Toast: 'Đã tạo 5 câu hỏi!'</t>
         </is>
       </c>
       <c r="I6" s="3" t="inlineStr">
@@ -755,12 +755,12 @@
       </c>
       <c r="K6" s="4" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="L6" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"> | Run: 2026-04-18 12:25 | Run: 2026-04-20 09:51 | Run: 2026-04-20 10:03</t>
+          <t xml:space="preserve"> | Run: 2026-04-18 12:25 | Run: 2026-04-20 09:51 | Run: 2026-04-20 10:03 | Run: 2026-04-21 13:38 | Run: 2026-04-21 13:50 | Run: 2026-04-21 15:11</t>
         </is>
       </c>
     </row>
@@ -822,7 +822,7 @@
       </c>
       <c r="L7" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve"> | Run: 2026-04-18 12:25 | Run: 2026-04-20 10:04</t>
+          <t xml:space="preserve"> | Run: 2026-04-18 12:25 | Run: 2026-04-20 10:04 | Run: 2026-04-21 15:13</t>
         </is>
       </c>
     </row>
@@ -864,12 +864,12 @@
       </c>
       <c r="H8" s="3" t="inlineStr">
         <is>
-          <t>Could not reach Questions step (URL: https://datn-quizapp.web.app/creator/new)</t>
+          <t>Generate button disabled on empty prompt: True; classes: px-6 py-3 bg-gradient-to-r from-purple-600 to-blue-600 hover:from-purple-700 hov</t>
         </is>
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>No API call made (button disabled — client-side validation)</t>
         </is>
       </c>
       <c r="J8" s="3" t="inlineStr">
@@ -879,12 +879,12 @@
       </c>
       <c r="K8" s="4" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="L8" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"> | Run: 2026-04-18 12:25 | Run: 2026-04-20 10:05</t>
+          <t xml:space="preserve"> | Run: 2026-04-18 12:25 | Run: 2026-04-20 10:05 | Run: 2026-04-21 15:22</t>
         </is>
       </c>
     </row>
@@ -926,12 +926,12 @@
       </c>
       <c r="H9" s="5" t="inlineStr">
         <is>
-          <t>Could not reach Questions step (URL: https://datn-quizapp.web.app/creator/new)</t>
+          <t>Toast (client validation): 'Đã tạo 5 câu hỏi!'; Blocked before API: True</t>
         </is>
       </c>
       <c r="I9" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>No API call made</t>
         </is>
       </c>
       <c r="J9" s="5" t="inlineStr">
@@ -941,12 +941,12 @@
       </c>
       <c r="K9" s="4" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="L9" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve"> | Run: 2026-04-18 12:25 | Run: 2026-04-20 10:07</t>
+          <t xml:space="preserve"> | Run: 2026-04-18 12:25 | Run: 2026-04-20 10:07 | Run: 2026-04-21 15:25</t>
         </is>
       </c>
     </row>
@@ -958,7 +958,7 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Request 30 questions → JSON parse failure</t>
+          <t>Request 30 questions (max valid, range 1-30) -&gt; exactly 30 generated in preview</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
@@ -983,32 +983,28 @@
       </c>
       <c r="G10" s="3" t="inlineStr">
         <is>
-          <t>Error shown in UI; not 30 questions generated</t>
+          <t>Exactly 30 question cards in preview; toast shows success</t>
         </is>
       </c>
       <c r="H10" s="3" t="inlineStr">
         <is>
-          <t>Could not reach Questions step (URL: https://datn-quizapp.web.app/creator/new)</t>
+          <t>Requested 30; preview shows 30 question card(s). Toast: 'Đã tạo 30 câu hỏi!'</t>
         </is>
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="J10" s="3" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
+          <t>Generated 30 questions (expected 30). CORRECT</t>
+        </is>
+      </c>
+      <c r="J10" s="3" t="n"/>
       <c r="K10" s="4" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="L10" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"> | Run: 2026-04-18 12:26 | Run: 2026-04-20 10:09</t>
+          <t xml:space="preserve"> | Run: 2026-04-18 12:26 | Run: 2026-04-20 10:09 | Run: 2026-04-21 15:33 | Run: 2026-04-21 15:48</t>
         </is>
       </c>
     </row>
@@ -1050,12 +1046,12 @@
       </c>
       <c r="H11" s="5" t="inlineStr">
         <is>
-          <t>Could not reach Questions step (URL: https://datn-quizapp.web.app/creator/new)</t>
+          <t>Requested 20; preview shows 20 card(s). Toast: 'Đã tạo 20 câu hỏi!'</t>
         </is>
       </c>
       <c r="I11" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Preview count=20 (expected 20). CORRECT</t>
         </is>
       </c>
       <c r="J11" s="5" t="inlineStr">
@@ -1065,12 +1061,12 @@
       </c>
       <c r="K11" s="4" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="L11" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve"> | Run: 2026-04-18 12:26 | Run: 2026-04-20 10:11</t>
+          <t xml:space="preserve"> | Run: 2026-04-18 12:26 | Run: 2026-04-20 10:11 | Run: 2026-04-21 15:51</t>
         </is>
       </c>
     </row>
@@ -1194,7 +1190,7 @@
       </c>
       <c r="L13" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve"> | Run: 2026-04-18 12:26 | Run: 2026-04-20 10:13</t>
+          <t xml:space="preserve"> | Run: 2026-04-18 12:26 | Run: 2026-04-20 10:13 | Run: 2026-04-21 15:54</t>
         </is>
       </c>
     </row>
@@ -1236,12 +1232,12 @@
       </c>
       <c r="H14" s="3" t="inlineStr">
         <is>
-          <t>Could not reach Questions step (URL: https://datn-quizapp.web.app/creator/new)</t>
+          <t>Toast on zero types: 'Đã tạo 5 câu hỏi!'; Preview opened: True</t>
         </is>
       </c>
       <c r="I14" s="3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>No DB write expected (should be blocked before API call)</t>
         </is>
       </c>
       <c r="J14" s="3" t="inlineStr">
@@ -1256,7 +1252,7 @@
       </c>
       <c r="L14" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"> | Run: 2026-04-18 12:26 | Run: 2026-04-20 10:15</t>
+          <t xml:space="preserve"> | Run: 2026-04-18 12:26 | Run: 2026-04-20 10:15 | Run: 2026-04-21 16:17</t>
         </is>
       </c>
     </row>
@@ -1298,12 +1294,12 @@
       </c>
       <c r="H15" s="5" t="inlineStr">
         <is>
-          <t>Could not reach Questions step (URL: https://datn-quizapp.web.app/creator/new)</t>
+          <t>Preview shows 5 question card(s). Toast: 'Đã tạo 5 câu hỏi!'</t>
         </is>
       </c>
       <c r="I15" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Found 5 question cards with text visible in preview</t>
         </is>
       </c>
       <c r="J15" s="5" t="inlineStr">
@@ -1313,12 +1309,12 @@
       </c>
       <c r="K15" s="4" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="L15" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve"> | Run: 2026-04-18 12:27 | Run: 2026-04-20 10:16</t>
+          <t xml:space="preserve"> | Run: 2026-04-18 12:27 | Run: 2026-04-20 10:16 | Run: 2026-04-21 16:24</t>
         </is>
       </c>
     </row>
@@ -1539,7 +1535,9 @@
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>Response: ''</t>
+          <t>Response: 'Hmmm, câu hỏi này không có trong các tài liệu bạn cung cấp. Tuy nhiên, mình có thể giúp bạn trả lời dựa trên kiến thức chung nhé! 😉
+Thủ đô của Pháp là **Paris**. 🇫🇷
+Paris không chỉ là thủ đô mà còn '</t>
         </is>
       </c>
       <c r="J6" s="4" t="inlineStr">
@@ -1549,7 +1547,7 @@
       </c>
       <c r="K6" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"> | Run: 2026-04-20 10:22</t>
+          <t xml:space="preserve"> | Run: 2026-04-20 10:22 | Run: 2026-04-21 16:29 | Run: 2026-04-21 16:36</t>
         </is>
       </c>
     </row>
@@ -1606,7 +1604,7 @@
       </c>
       <c r="K7" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve"> | Run: 2026-04-20 10:24</t>
+          <t xml:space="preserve"> | Run: 2026-04-20 10:24 | Run: 2026-04-21 16:38</t>
         </is>
       </c>
     </row>
@@ -1653,7 +1651,9 @@
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>Response (0 chars): ''</t>
+          <t>Response (695 chars): 'Để hiểu bối cảnh lịch sử Pháp xâm chiếm Việt Nam, chúng ta cần nhìn lại thời điểm đó nhé! 🇫🇷🇻🇳
+Pháp nổ súng tấn công Việt Nam lần đầu tiên vào năm **1858** [1]. Đây là sự kiện mở đầu cho quá trình xâm lược kéo dài của thực dân Pháp.
+Sau nhiều năm chiến tranh và thương lượng, Pháp đã từng bước thiế'</t>
         </is>
       </c>
       <c r="J8" s="4" t="inlineStr">
@@ -1663,7 +1663,7 @@
       </c>
       <c r="K8" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"> | Run: 2026-04-20 10:26</t>
+          <t xml:space="preserve"> | Run: 2026-04-20 10:26 | Run: 2026-04-21 16:41 | Run: 2026-04-21 17:01</t>
         </is>
       </c>
     </row>
@@ -1710,7 +1710,11 @@
       </c>
       <c r="I9" s="5" t="inlineStr">
         <is>
-          <t>Response to 'a': ''; Known '0' bug: False</t>
+          <t>Response to 'a': '🤔 Mình chưa hiểu rõ. Bạn có thể nói cụ thể hơn không?
+💡 **Gợi ý:**
+- Tìm quiz: "Quiz về JavaScript"
+- Học lộ trình: "Tôi muốn học Web Development"
+- Hỏi kiến thức: "React là gì?"'; Known '0' bug: False</t>
         </is>
       </c>
       <c r="J9" s="4" t="inlineStr">
@@ -1720,7 +1724,7 @@
       </c>
       <c r="K9" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve"> | Run: 2026-04-20 10:28</t>
+          <t xml:space="preserve"> | Run: 2026-04-20 10:28 | Run: 2026-04-21 17:03</t>
         </is>
       </c>
     </row>
@@ -1765,13 +1769,23 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="I10" s="3" t="n"/>
+      <c r="I10" s="3" t="inlineStr">
+        <is>
+          <t>Response to 2001-char input: '[ERROR] Đã xảy ra lỗi
+Đã xảy ra lỗi. Vui lòng thử lại sau.
+Thử lại'</t>
+        </is>
+      </c>
       <c r="J10" s="4" t="inlineStr">
         <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="K10" s="3" t="n"/>
+          <t>Vague error or fallback shown</t>
+        </is>
+      </c>
+      <c r="K10" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> | Run: 2026-04-21 17:12</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="25.5" customHeight="1">
       <c r="A11" s="5" t="inlineStr">
@@ -1816,7 +1830,10 @@
       </c>
       <c r="I11" s="5" t="inlineStr">
         <is>
-          <t>Response (0 chars): ''</t>
+          <t>Response (815 chars): 'Chào bạn! 👋 Quiz "Chuyên gia Thể thao: Lịch sử, Chiến thuật &amp; Kỹ thuật" là một bài kiểm tra thú vị dành cho những người yêu thể thao thực thụ 🏆.
+Nội dung quiz bao gồm các kiến thức chuyên sâu về:
+*   **Lịch sử thể thao:** Tìm hiểu về những cột mốc quan trọng, ví dụ như lịch sử World Cup 🌍.
+*   **C'</t>
         </is>
       </c>
       <c r="J11" s="4" t="inlineStr">
@@ -1826,7 +1843,7 @@
       </c>
       <c r="K11" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve"> | Run: 2026-04-20 10:31</t>
+          <t xml:space="preserve"> | Run: 2026-04-20 10:31 | Run: 2026-04-21 17:14</t>
         </is>
       </c>
     </row>
@@ -1873,7 +1890,10 @@
       </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>Response: ''</t>
+          <t>Response: 'Hiện tại, mình chưa có bất kỳ quiz nào liên quan đến tiếng Nga bạn nhé. 🇷🇺
+Quiz mà mình có chủ yếu tập trung vào các lĩnh vực như:
+*   **Lập trình AI và tạo quiz:** Giúp bạn kiểm tra kiến thức về AI, cách tạo câu hỏi, v.v. 🤖💡
+*   **Phát triển web:** Bao gồm các chủ đề về frontend, backend, HTML, C'</t>
         </is>
       </c>
       <c r="J12" s="4" t="inlineStr">
@@ -1883,7 +1903,7 @@
       </c>
       <c r="K12" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"> | Run: 2026-04-20 10:34</t>
+          <t xml:space="preserve"> | Run: 2026-04-20 10:34 | Run: 2026-04-21 17:19</t>
         </is>
       </c>
     </row>
@@ -1928,13 +1948,24 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="I13" s="5" t="n"/>
+      <c r="I13" s="5" t="inlineStr">
+        <is>
+          <t>Turn1: 'Chào bạn! 👋 Mình có thể giúp bạn tìm các bài quiz về lịch sử. Dựa vào thông tin bạn cung cấp, mình thấy có các bài quiz sau:
+*   **Thử thách Lịch sử ' | Turn2: 'Chào bạn! 😊 Dưới đây là **5 quiz phổ biến** trên hệ thống:
+📊 **Các danh mục nổi bật:** Sports, Science, Programming
+🎯 Chọn quiz bạn quan tâm để bắt '</t>
+        </is>
+      </c>
       <c r="J13" s="4" t="inlineStr">
         <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="K13" s="5" t="n"/>
+          <t>Context maintained across turns: True</t>
+        </is>
+      </c>
+      <c r="K13" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> | Run: 2026-04-21 17:37</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
@@ -1979,7 +2010,9 @@
       </c>
       <c r="I14" s="3" t="inlineStr">
         <is>
-          <t>Response to 'lo den la gi': ''</t>
+          <t>Response to 'lo den la gi': 'Logarit là phép toán ngược của **lũy thừa** 🧮.
+Nói một cách dễ hiểu, nếu bạn có một phép tính lũy thừa, ví dụ $2^3 = 8$, thì logarit sẽ giúp bạn tìm ra số mũ. Logarit cơ số 2 của 8 là 3, ký hiệu là $\log_2 8 = 3$ 💡.
+Nó giống như bạn biết kết quả của một phép nhân và muốn tìm xem hai số nào đã nhân'</t>
         </is>
       </c>
       <c r="J14" s="4" t="inlineStr">
@@ -1989,7 +2022,7 @@
       </c>
       <c r="K14" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"> | Run: 2026-04-20 10:38</t>
+          <t xml:space="preserve"> | Run: 2026-04-20 10:38 | Run: 2026-04-21 17:50</t>
         </is>
       </c>
     </row>
@@ -2046,7 +2079,7 @@
       </c>
       <c r="K15" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve"> | Run: 2026-04-20 10:39</t>
+          <t xml:space="preserve"> | Run: 2026-04-20 10:39 | Run: 2026-04-21 17:53</t>
         </is>
       </c>
     </row>
@@ -2093,7 +2126,8 @@
       </c>
       <c r="I16" s="3" t="inlineStr">
         <is>
-          <t>Raw Markdown visible: False; Rendered HTML elements present: False; Snippet: ''</t>
+          <t>Raw Markdown visible: True; Rendered HTML elements present: False; Snippet: 'Vụ nổ Big Bang là **mô hình khoa học giải thích sự hình thành và tiến hóa của vũ trụ** 💥.
+Theo thuyết này, vũ trụ của chúng ta bắt đầu từ một **điểm kỳ dị** 🤏 (một điểm cực nhỏ, nóng và đặc) và sau đ'</t>
         </is>
       </c>
       <c r="J16" s="4" t="inlineStr">
@@ -2103,7 +2137,7 @@
       </c>
       <c r="K16" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"> | Run: 2026-04-20 10:41</t>
+          <t xml:space="preserve"> | Run: 2026-04-20 10:41 | Run: 2026-04-21 17:57</t>
         </is>
       </c>
     </row>
@@ -2150,7 +2184,7 @@
       </c>
       <c r="I17" s="5" t="inlineStr">
         <is>
-          <t>Response appeared in 642.9s (threshold: 10s)</t>
+          <t>Response appeared in 38.7s (threshold: 10s)</t>
         </is>
       </c>
       <c r="J17" s="4" t="inlineStr">
@@ -2160,7 +2194,7 @@
       </c>
       <c r="K17" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve"> | Run: 2026-04-20 10:53</t>
+          <t xml:space="preserve"> | Run: 2026-04-20 10:53 | Run: 2026-04-21 18:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: add AI generator and chatbot Selenium test suite with supporting Excel data file
</commit_message>
<xml_diff>
--- a/data/TC_AIFeatures.xlsx
+++ b/data/TC_AIFeatures.xlsx
@@ -1473,7 +1473,7 @@
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>Rollback</t>
+          <t>Actual DB</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
@@ -1530,7 +1530,7 @@
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>No DB state created</t>
         </is>
       </c>
       <c r="I6" s="3" t="inlineStr">
@@ -1542,7 +1542,7 @@
       </c>
       <c r="J6" s="4" t="inlineStr">
         <is>
-          <t>No DB state created</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="K6" s="3" t="inlineStr">
@@ -1589,7 +1589,7 @@
       </c>
       <c r="H7" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>No API call triggered</t>
         </is>
       </c>
       <c r="I7" s="5" t="inlineStr">
@@ -1599,7 +1599,7 @@
       </c>
       <c r="J7" s="4" t="inlineStr">
         <is>
-          <t>No API call triggered</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="K7" s="5" t="inlineStr">
@@ -1646,7 +1646,7 @@
       </c>
       <c r="H8" s="3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Citations found: False</t>
         </is>
       </c>
       <c r="I8" s="3" t="inlineStr">
@@ -1658,7 +1658,7 @@
       </c>
       <c r="J8" s="4" t="inlineStr">
         <is>
-          <t>Citations found: False</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="K8" s="3" t="inlineStr">
@@ -1705,7 +1705,7 @@
       </c>
       <c r="H9" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>No crash; no hallucination</t>
         </is>
       </c>
       <c r="I9" s="5" t="inlineStr">
@@ -1719,7 +1719,7 @@
       </c>
       <c r="J9" s="4" t="inlineStr">
         <is>
-          <t>No crash; no hallucination</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="K9" s="5" t="inlineStr">
@@ -1766,7 +1766,7 @@
       </c>
       <c r="H10" s="3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Vague error or fallback shown</t>
         </is>
       </c>
       <c r="I10" s="3" t="inlineStr">
@@ -1778,7 +1778,7 @@
       </c>
       <c r="J10" s="4" t="inlineStr">
         <is>
-          <t>Vague error or fallback shown</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="K10" s="3" t="inlineStr">
@@ -1825,7 +1825,7 @@
       </c>
       <c r="H11" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Citations found: False</t>
         </is>
       </c>
       <c r="I11" s="5" t="inlineStr">
@@ -1838,7 +1838,7 @@
       </c>
       <c r="J11" s="4" t="inlineStr">
         <is>
-          <t>Citations found: False</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="K11" s="5" t="inlineStr">
@@ -1885,7 +1885,7 @@
       </c>
       <c r="H12" s="3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>No session state written</t>
         </is>
       </c>
       <c r="I12" s="3" t="inlineStr">
@@ -1898,7 +1898,7 @@
       </c>
       <c r="J12" s="4" t="inlineStr">
         <is>
-          <t>No session state written</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="K12" s="3" t="inlineStr">
@@ -1945,7 +1945,7 @@
       </c>
       <c r="H13" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Context maintained across turns: True</t>
         </is>
       </c>
       <c r="I13" s="5" t="inlineStr">
@@ -1958,7 +1958,7 @@
       </c>
       <c r="J13" s="4" t="inlineStr">
         <is>
-          <t>Context maintained across turns: True</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="K13" s="5" t="inlineStr">
@@ -2005,7 +2005,7 @@
       </c>
       <c r="H14" s="3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Diacritic-insensitive retrieval successful: False</t>
         </is>
       </c>
       <c r="I14" s="3" t="inlineStr">
@@ -2017,7 +2017,7 @@
       </c>
       <c r="J14" s="4" t="inlineStr">
         <is>
-          <t>Diacritic-insensitive retrieval successful: False</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="K14" s="3" t="inlineStr">
@@ -2064,7 +2064,7 @@
       </c>
       <c r="H15" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>N/A – UI-only streaming indicator check</t>
         </is>
       </c>
       <c r="I15" s="5" t="inlineStr">
@@ -2074,7 +2074,7 @@
       </c>
       <c r="J15" s="4" t="inlineStr">
         <is>
-          <t>N/A – UI-only streaming indicator check</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="K15" s="5" t="inlineStr">
@@ -2121,7 +2121,7 @@
       </c>
       <c r="H16" s="3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>N/A – UI-only rendering check</t>
         </is>
       </c>
       <c r="I16" s="3" t="inlineStr">
@@ -2132,7 +2132,7 @@
       </c>
       <c r="J16" s="4" t="inlineStr">
         <is>
-          <t>N/A – UI-only rendering check</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="K16" s="3" t="inlineStr">
@@ -2179,7 +2179,7 @@
       </c>
       <c r="H17" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Performance within threshold</t>
         </is>
       </c>
       <c r="I17" s="5" t="inlineStr">
@@ -2189,7 +2189,7 @@
       </c>
       <c r="J17" s="4" t="inlineStr">
         <is>
-          <t>Performance within threshold</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="K17" s="5" t="inlineStr">

</xml_diff>

<commit_message>
feat: implement Selenium test suite for AI features and quiz management with supporting documentation and test data
</commit_message>
<xml_diff>
--- a/data/TC_AIFeatures.xlsx
+++ b/data/TC_AIFeatures.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="34452" yWindow="1188" windowWidth="30936" windowHeight="16776" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="5370" yWindow="3390" windowWidth="28800" windowHeight="15370" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="TC_AIGenerator" sheetId="1" state="visible" r:id="rId1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -48,8 +48,41 @@
       <color rgb="FF9C6500"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <family val="2"/>
+      <color theme="1"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <family val="2"/>
+      <b val="1"/>
+      <color rgb="FF276221"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <family val="2"/>
+      <color theme="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <family val="2"/>
+      <b val="1"/>
+      <color rgb="FF7B5E00"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <family val="2"/>
+      <b val="1"/>
+      <color rgb="FF9C0006"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="12">
     <fill>
       <patternFill/>
     </fill>
@@ -81,8 +114,38 @@
         <fgColor rgb="FFEBF3FB"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F7FC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="6">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -130,6 +193,66 @@
       <diagonal/>
     </border>
     <border>
+      <left style="medium">
+        <color rgb="FFBFBFBF"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFBFBFBF"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFBFBFBF"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFBFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFBFBFBF"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFBFBFBF"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFBFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFBFBFBF"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFBFBFBF"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFBFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFBFBFBF"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFBFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left/>
       <right/>
       <top style="thin">
@@ -153,7 +276,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -171,9 +294,48 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="10" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="11" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Bình thường" xfId="0" builtinId="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -536,8 +698,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L15"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
+  <dimension ref="A1:N15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="36" customWidth="1" min="2" max="2"/>
@@ -573,6 +735,8 @@
       <c r="J1" s="7" t="n"/>
       <c r="K1" s="7" t="n"/>
       <c r="L1" s="8" t="n"/>
+      <c r="M1" s="7" t="n"/>
+      <c r="N1" s="8" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
@@ -595,6 +759,8 @@
       <c r="J2" s="7" t="n"/>
       <c r="K2" s="7" t="n"/>
       <c r="L2" s="8" t="n"/>
+      <c r="M2" s="7" t="n"/>
+      <c r="N2" s="8" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
@@ -617,6 +783,8 @@
       <c r="J3" s="7" t="n"/>
       <c r="K3" s="7" t="n"/>
       <c r="L3" s="8" t="n"/>
+      <c r="M3" s="7" t="n"/>
+      <c r="N3" s="8" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
@@ -639,8 +807,10 @@
       <c r="J4" s="7" t="n"/>
       <c r="K4" s="7" t="n"/>
       <c r="L4" s="8" t="n"/>
-    </row>
-    <row r="5" ht="27.75" customHeight="1">
+      <c r="M4" s="7" t="n"/>
+      <c r="N4" s="8" t="n"/>
+    </row>
+    <row r="5" ht="27.75" customHeight="1" thickBot="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
           <t>TC_ID</t>
@@ -691,632 +861,618 @@
           <t>Rollback</t>
         </is>
       </c>
-      <c r="K5" s="2" t="inlineStr">
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Actual UI</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>Actual DB</t>
+        </is>
+      </c>
+      <c r="M5" s="2" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="L5" s="2" t="inlineStr">
+      <c r="N5" s="2" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="25.5" customHeight="1">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>TC-GEN-001</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="inlineStr">
+    <row r="6" ht="25.5" customHeight="1" thickBot="1">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>TC-AQZ-001</t>
+        </is>
+      </c>
+      <c r="B6" s="10" t="inlineStr">
         <is>
           <t>Valid text prompt → generate 5 MCQ</t>
         </is>
       </c>
-      <c r="C6" s="3" t="inlineStr">
+      <c r="C6" s="10" t="inlineStr">
         <is>
           <t>CREATOR</t>
         </is>
       </c>
-      <c r="D6" s="3" t="inlineStr">
+      <c r="D6" s="10" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E6" s="3" t="inlineStr">
+      <c r="E6" s="10" t="inlineStr">
         <is>
           <t>Tạo câu hỏi về lịch sử Việt Nam</t>
         </is>
       </c>
-      <c r="F6" s="3" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="G6" s="3" t="inlineStr">
+      <c r="F6" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="G6" s="10" t="inlineStr">
         <is>
           <t>5 questions generated; preview shown</t>
         </is>
       </c>
-      <c r="H6" s="3" t="inlineStr">
+      <c r="H6" s="10" t="inlineStr">
         <is>
           <t>Preview shows 5 question card(s). Toast: 'Đã tạo 5 câu hỏi!'</t>
         </is>
       </c>
-      <c r="I6" s="3" t="inlineStr">
+      <c r="I6" s="10" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="J6" s="3" t="inlineStr">
+      <c r="J6" s="10" t="inlineStr">
         <is>
           <t>Delete generated quiz</t>
         </is>
       </c>
-      <c r="K6" s="4" t="inlineStr">
+      <c r="M6" s="11" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="L6" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> | Run: 2026-04-18 12:25 | Run: 2026-04-20 09:51 | Run: 2026-04-20 10:03 | Run: 2026-04-21 13:38 | Run: 2026-04-21 13:50 | Run: 2026-04-21 15:11</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="5" t="inlineStr">
-        <is>
-          <t>TC-GEN-002</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="inlineStr">
+      <c r="N6" s="12" t="n"/>
+    </row>
+    <row r="7" ht="46.5" customHeight="1" thickBot="1">
+      <c r="A7" s="13" t="inlineStr">
+        <is>
+          <t>TC-AQZ-002</t>
+        </is>
+      </c>
+      <c r="B7" s="14" t="inlineStr">
+        <is>
+          <t>Empty prompt → validation error</t>
+        </is>
+      </c>
+      <c r="C7" s="14" t="inlineStr">
+        <is>
+          <t>CREATOR</t>
+        </is>
+      </c>
+      <c r="D7" s="14" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E7" s="14" t="inlineStr">
+        <is>
+          <t>(empty)</t>
+        </is>
+      </c>
+      <c r="F7" s="14" t="n">
+        <v>5</v>
+      </c>
+      <c r="G7" s="14" t="inlineStr">
+        <is>
+          <t>Validation error; send button disabled or error shown</t>
+        </is>
+      </c>
+      <c r="H7" s="14" t="inlineStr">
+        <is>
+          <t>Generate button disabled on empty prompt: True; classes: px-6 py-3 bg-gradient-to-r from-purple-600 to-blue-600 hover:from-purple-700 hov</t>
+        </is>
+      </c>
+      <c r="I7" s="14" t="inlineStr">
+        <is>
+          <t>No API call made (button disabled — client-side validation)</t>
+        </is>
+      </c>
+      <c r="J7" s="14" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="M7" s="15" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="N7" s="16" t="n"/>
+    </row>
+    <row r="8" ht="25.5" customHeight="1" thickBot="1">
+      <c r="A8" s="17" t="inlineStr">
+        <is>
+          <t>TC-AQZ-004</t>
+        </is>
+      </c>
+      <c r="B8" s="18" t="inlineStr">
         <is>
           <t>Valid PDF file → generate questions</t>
         </is>
       </c>
-      <c r="C7" s="5" t="inlineStr">
+      <c r="C8" s="18" t="inlineStr">
         <is>
           <t>CREATOR</t>
         </is>
       </c>
-      <c r="D7" s="5" t="inlineStr">
+      <c r="D8" s="18" t="inlineStr">
         <is>
           <t>PDF</t>
         </is>
       </c>
-      <c r="E7" s="5" t="inlineStr">
+      <c r="E8" s="18" t="inlineStr">
         <is>
           <t>data/sample_pdf_valid.pdf</t>
         </is>
       </c>
-      <c r="F7" s="5" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="G7" s="5" t="inlineStr">
+      <c r="F8" s="18" t="n">
+        <v>5</v>
+      </c>
+      <c r="G8" s="18" t="inlineStr">
         <is>
           <t>Questions generated from PDF content</t>
         </is>
       </c>
-      <c r="H7" s="5" t="inlineStr">
-        <is>
-          <t>Sample PDF not found at C:\quiz-trivia-tooltest\data\sample_pdf_valid.pdf — place a valid PDF there to run this TC</t>
-        </is>
-      </c>
-      <c r="I7" s="5" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="J7" s="5" t="inlineStr">
+      <c r="H8" s="18" t="inlineStr">
+        <is>
+          <t>Questions generated from PDF content; preview shows question cards</t>
+        </is>
+      </c>
+      <c r="I8" s="18" t="inlineStr">
+        <is>
+          <t>TIMEOUT: file selected via Selenium send_keys but Generate button stayed disabled — likely React onChange not triggered; try clicking 'Select File' manually to confirm</t>
+        </is>
+      </c>
+      <c r="J8" s="18" t="inlineStr">
         <is>
           <t>Delete</t>
         </is>
       </c>
-      <c r="K7" s="4" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="L7" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> | Run: 2026-04-18 12:25 | Run: 2026-04-20 10:04 | Run: 2026-04-21 15:13</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="25.5" customHeight="1">
-      <c r="A8" s="3" t="inlineStr">
-        <is>
-          <t>TC-GEN-003</t>
-        </is>
-      </c>
-      <c r="B8" s="3" t="inlineStr">
-        <is>
-          <t>Empty prompt → validation error</t>
-        </is>
-      </c>
-      <c r="C8" s="3" t="inlineStr">
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>Generate button did not become clickable after file upload (React state not updated)</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>TIMEOUT: file selected via Selenium send_keys but Generate button stayed disabled — likely React onChange not triggered; try clicking 'Select File' manually to confirm</t>
+        </is>
+      </c>
+      <c r="M8" s="19" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="N8" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> | Run: 2026-05-05 16:56 | Run: 2026-05-05 17:08 | Run: 2026-05-05 17:21 | Run: 2026-05-05 17:41 | Run: 2026-05-05 17:56</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="409.5" customHeight="1" thickBot="1">
+      <c r="A9" s="17" t="inlineStr">
+        <is>
+          <t>TC-AQZ-009</t>
+        </is>
+      </c>
+      <c r="B9" s="18" t="inlineStr">
+        <is>
+          <t>Valid prompt → verify question schema</t>
+        </is>
+      </c>
+      <c r="C9" s="18" t="inlineStr">
         <is>
           <t>CREATOR</t>
         </is>
       </c>
-      <c r="D8" s="3" t="inlineStr">
+      <c r="D9" s="18" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E8" s="3" t="inlineStr">
-        <is>
-          <t>(empty)</t>
-        </is>
-      </c>
-      <c r="F8" s="3" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="G8" s="3" t="inlineStr">
-        <is>
-          <t>Validation error; send button disabled or error shown</t>
-        </is>
-      </c>
-      <c r="H8" s="3" t="inlineStr">
-        <is>
-          <t>Generate button disabled on empty prompt: True; classes: px-6 py-3 bg-gradient-to-r from-purple-600 to-blue-600 hover:from-purple-700 hov</t>
-        </is>
-      </c>
-      <c r="I8" s="3" t="inlineStr">
-        <is>
-          <t>No API call made (button disabled — client-side validation)</t>
-        </is>
-      </c>
-      <c r="J8" s="3" t="inlineStr">
+      <c r="E9" s="18" t="inlineStr">
+        <is>
+          <t>Câu hỏi về công nghệ thông tin</t>
+        </is>
+      </c>
+      <c r="F9" s="18" t="n">
+        <v>5</v>
+      </c>
+      <c r="G9" s="18" t="inlineStr">
+        <is>
+          <t>Questions shown with type, options, correct answer</t>
+        </is>
+      </c>
+      <c r="H9" s="18" t="inlineStr">
+        <is>
+          <t>Preview shows 5 question card(s). Toast: 'Đã tạo 5 câu hỏi!'</t>
+        </is>
+      </c>
+      <c r="I9" s="18" t="inlineStr">
+        <is>
+          <t>Found 5 question cards with text visible in preview</t>
+        </is>
+      </c>
+      <c r="J9" s="18" t="inlineStr">
+        <is>
+          <t>Delete</t>
+        </is>
+      </c>
+      <c r="M9" s="15" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="N9" s="20" t="n"/>
+    </row>
+    <row r="10" ht="25.5" customHeight="1" thickBot="1">
+      <c r="A10" s="17" t="inlineStr">
+        <is>
+          <t>TC-AQZ-010</t>
+        </is>
+      </c>
+      <c r="B10" s="18" t="inlineStr">
+        <is>
+          <t>User role blocked from AI Generator</t>
+        </is>
+      </c>
+      <c r="C10" s="18" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="D10" s="18" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E10" s="18" t="inlineStr">
+        <is>
+          <t>Tạo câu hỏi về lịch sử</t>
+        </is>
+      </c>
+      <c r="F10" s="18" t="n">
+        <v>5</v>
+      </c>
+      <c r="G10" s="18" t="inlineStr">
+        <is>
+          <t>Access denied; AI Generator not visible</t>
+        </is>
+      </c>
+      <c r="H10" s="18" t="inlineStr">
+        <is>
+          <t>USER navigated to /creator/new → landed at: https://datn-quizapp.web.app/creator/new</t>
+        </is>
+      </c>
+      <c r="I10" s="18" t="inlineStr">
+        <is>
+          <t>No data saved (USER role blocked from creator route); Firestore role='creator'</t>
+        </is>
+      </c>
+      <c r="J10" s="18" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="K8" s="4" t="inlineStr">
+      <c r="M10" s="21" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="N10" s="18" t="inlineStr">
+        <is>
+          <t>User role can access /creator/new route; should be blocked</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="35" customHeight="1" thickBot="1">
+      <c r="A11" s="13" t="inlineStr">
+        <is>
+          <t>TC-AQZ-011</t>
+        </is>
+      </c>
+      <c r="B11" s="14" t="inlineStr">
+        <is>
+          <t>Zero question types selected</t>
+        </is>
+      </c>
+      <c r="C11" s="14" t="inlineStr">
+        <is>
+          <t>CREATOR</t>
+        </is>
+      </c>
+      <c r="D11" s="14" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E11" s="14" t="inlineStr">
+        <is>
+          <t>Tạo câu hỏi về khoa học</t>
+        </is>
+      </c>
+      <c r="F11" s="14" t="n">
+        <v>5</v>
+      </c>
+      <c r="G11" s="14" t="inlineStr">
+        <is>
+          <t>Validation error; cannot submit</t>
+        </is>
+      </c>
+      <c r="H11" s="14" t="inlineStr">
+        <is>
+          <t>Toast on zero types: 'Đã tạo 5 câu hỏi!'; Preview opened: True</t>
+        </is>
+      </c>
+      <c r="I11" s="14" t="inlineStr">
+        <is>
+          <t>No DB write expected (should be blocked before API call)</t>
+        </is>
+      </c>
+      <c r="J11" s="14" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="M11" s="21" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="N11" s="14" t="inlineStr">
+        <is>
+          <t>Zero question types selected still generates 5 questions; no validation error</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="253.5" customHeight="1" thickBot="1">
+      <c r="A12" s="17" t="inlineStr">
+        <is>
+          <t>TC-AQZ-015</t>
+        </is>
+      </c>
+      <c r="B12" s="18" t="inlineStr">
+        <is>
+          <t>Prompt &gt; 2000 chars → no client guard</t>
+        </is>
+      </c>
+      <c r="C12" s="18" t="inlineStr">
+        <is>
+          <t>CREATOR</t>
+        </is>
+      </c>
+      <c r="D12" s="18" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E12" s="18" t="inlineStr">
+        <is>
+          <t>aaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaa…</t>
+        </is>
+      </c>
+      <c r="F12" s="18" t="n">
+        <v>5</v>
+      </c>
+      <c r="G12" s="18" t="inlineStr">
+        <is>
+          <t>No client-side block; error or token limit crash</t>
+        </is>
+      </c>
+      <c r="H12" s="18" t="inlineStr">
+        <is>
+          <t>Toast (client validation): 'Đã tạo 5 câu hỏi!'; Blocked before API: True</t>
+        </is>
+      </c>
+      <c r="I12" s="18" t="inlineStr">
+        <is>
+          <t>No API call made</t>
+        </is>
+      </c>
+      <c r="J12" s="18" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="M12" s="15" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="L8" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> | Run: 2026-04-18 12:25 | Run: 2026-04-20 10:05 | Run: 2026-04-21 15:22</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="409.5" customHeight="1">
-      <c r="A9" s="5" t="inlineStr">
-        <is>
-          <t>TC-GEN-004</t>
-        </is>
-      </c>
-      <c r="B9" s="5" t="inlineStr">
-        <is>
-          <t>Prompt &gt; 2000 chars → no client guard</t>
-        </is>
-      </c>
-      <c r="C9" s="5" t="inlineStr">
+      <c r="N12" s="20" t="n"/>
+    </row>
+    <row r="13" ht="35" customHeight="1" thickBot="1">
+      <c r="A13" s="13" t="inlineStr">
+        <is>
+          <t>TC-AQZ-017</t>
+        </is>
+      </c>
+      <c r="B13" s="14" t="inlineStr">
+        <is>
+          <t>File &gt; 5MB → no client guard</t>
+        </is>
+      </c>
+      <c r="C13" s="14" t="inlineStr">
         <is>
           <t>CREATOR</t>
         </is>
       </c>
-      <c r="D9" s="5" t="inlineStr">
+      <c r="D13" s="14" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="E13" s="14" t="inlineStr">
+        <is>
+          <t>data/sample_pdf_large.pdf</t>
+        </is>
+      </c>
+      <c r="F13" s="14" t="n">
+        <v>5</v>
+      </c>
+      <c r="G13" s="14" t="inlineStr">
+        <is>
+          <t>Error: file too large</t>
+        </is>
+      </c>
+      <c r="H13" s="14" t="inlineStr">
+        <is>
+          <t>Toast error: file too large (&gt;5MB); no questions generated</t>
+        </is>
+      </c>
+      <c r="I13" s="14" t="inlineStr">
+        <is>
+          <t>TIMEOUT: Generate button stayed disabled — React onChange may not have fired via send_keys</t>
+        </is>
+      </c>
+      <c r="J13" s="14" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>Generate button did not become clickable after large file upload</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>TIMEOUT: Generate button stayed disabled — React onChange may not have fired via send_keys</t>
+        </is>
+      </c>
+      <c r="M13" s="19" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="N13" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> | Run: 2026-05-05 17:27 | Run: 2026-05-05 17:45 | Run: 2026-05-05 17:53</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="23.5" customHeight="1" thickBot="1">
+      <c r="A14" s="17" t="inlineStr">
+        <is>
+          <t>TC-AQZ-019</t>
+        </is>
+      </c>
+      <c r="B14" s="18" t="inlineStr">
+        <is>
+          <t>Off-by-one: request 20 → 21 generated</t>
+        </is>
+      </c>
+      <c r="C14" s="18" t="inlineStr">
+        <is>
+          <t>CREATOR</t>
+        </is>
+      </c>
+      <c r="D14" s="18" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E9" s="5" t="inlineStr">
-        <is>
-          <t>aaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaa</t>
-        </is>
-      </c>
-      <c r="F9" s="5" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="G9" s="5" t="inlineStr">
-        <is>
-          <t>No client-side block; error or token limit crash</t>
-        </is>
-      </c>
-      <c r="H9" s="5" t="inlineStr">
-        <is>
-          <t>Toast (client validation): 'Đã tạo 5 câu hỏi!'; Blocked before API: True</t>
-        </is>
-      </c>
-      <c r="I9" s="5" t="inlineStr">
-        <is>
-          <t>No API call made</t>
-        </is>
-      </c>
-      <c r="J9" s="5" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="K9" s="4" t="inlineStr">
+      <c r="E14" s="18" t="inlineStr">
+        <is>
+          <t>Tạo câu hỏi về toán học</t>
+        </is>
+      </c>
+      <c r="F14" s="18" t="n">
+        <v>20</v>
+      </c>
+      <c r="G14" s="18" t="inlineStr">
+        <is>
+          <t>Preview shows 20 questions</t>
+        </is>
+      </c>
+      <c r="H14" s="18" t="inlineStr">
+        <is>
+          <t>Requested 20; preview shows 20 card(s). Toast: 'Đã tạo 20 câu hỏi!'</t>
+        </is>
+      </c>
+      <c r="I14" s="18" t="inlineStr">
+        <is>
+          <t>Preview count=20 (expected 20). CORRECT</t>
+        </is>
+      </c>
+      <c r="J14" s="18" t="inlineStr">
+        <is>
+          <t>Delete</t>
+        </is>
+      </c>
+      <c r="M14" s="15" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="L9" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> | Run: 2026-04-18 12:25 | Run: 2026-04-20 10:07 | Run: 2026-04-21 15:25</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="25.5" customHeight="1">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>TC-GEN-005</t>
-        </is>
-      </c>
-      <c r="B10" s="3" t="inlineStr">
+      <c r="N14" s="20" t="n"/>
+    </row>
+    <row r="15" ht="25.5" customHeight="1" thickBot="1">
+      <c r="A15" s="13" t="inlineStr">
+        <is>
+          <t>TC-AQZ-020</t>
+        </is>
+      </c>
+      <c r="B15" s="14" t="inlineStr">
         <is>
           <t>Request 30 questions (max valid, range 1-30) -&gt; exactly 30 generated in preview</t>
         </is>
       </c>
-      <c r="C10" s="3" t="inlineStr">
+      <c r="C15" s="14" t="inlineStr">
         <is>
           <t>CREATOR</t>
         </is>
       </c>
-      <c r="D10" s="3" t="inlineStr">
+      <c r="D15" s="14" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E10" s="3" t="inlineStr">
+      <c r="E15" s="14" t="inlineStr">
         <is>
           <t>Tạo câu hỏi về địa lý thế giới</t>
         </is>
       </c>
-      <c r="F10" s="3" t="inlineStr">
-        <is>
-          <t>30</t>
-        </is>
-      </c>
-      <c r="G10" s="3" t="inlineStr">
+      <c r="F15" s="14" t="n">
+        <v>30</v>
+      </c>
+      <c r="G15" s="14" t="inlineStr">
         <is>
           <t>Exactly 30 question cards in preview; toast shows success</t>
         </is>
       </c>
-      <c r="H10" s="3" t="inlineStr">
+      <c r="H15" s="14" t="inlineStr">
         <is>
           <t>Requested 30; preview shows 30 question card(s). Toast: 'Đã tạo 30 câu hỏi!'</t>
         </is>
       </c>
-      <c r="I10" s="3" t="inlineStr">
+      <c r="I15" s="14" t="inlineStr">
         <is>
           <t>Generated 30 questions (expected 30). CORRECT</t>
         </is>
       </c>
-      <c r="J10" s="3" t="n"/>
-      <c r="K10" s="4" t="inlineStr">
+      <c r="J15" s="16" t="n"/>
+      <c r="M15" s="15" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="L10" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> | Run: 2026-04-18 12:26 | Run: 2026-04-20 10:09 | Run: 2026-04-21 15:33 | Run: 2026-04-21 15:48</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="5" t="inlineStr">
-        <is>
-          <t>TC-GEN-006</t>
-        </is>
-      </c>
-      <c r="B11" s="5" t="inlineStr">
-        <is>
-          <t>Off-by-one: request 20 → 21 generated</t>
-        </is>
-      </c>
-      <c r="C11" s="5" t="inlineStr">
-        <is>
-          <t>CREATOR</t>
-        </is>
-      </c>
-      <c r="D11" s="5" t="inlineStr">
-        <is>
-          <t>Text</t>
-        </is>
-      </c>
-      <c r="E11" s="5" t="inlineStr">
-        <is>
-          <t>Tạo câu hỏi về toán học</t>
-        </is>
-      </c>
-      <c r="F11" s="5" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
-      </c>
-      <c r="G11" s="5" t="inlineStr">
-        <is>
-          <t>Preview shows 20 questions</t>
-        </is>
-      </c>
-      <c r="H11" s="5" t="inlineStr">
-        <is>
-          <t>Requested 20; preview shows 20 card(s). Toast: 'Đã tạo 20 câu hỏi!'</t>
-        </is>
-      </c>
-      <c r="I11" s="5" t="inlineStr">
-        <is>
-          <t>Preview count=20 (expected 20). CORRECT</t>
-        </is>
-      </c>
-      <c r="J11" s="5" t="inlineStr">
-        <is>
-          <t>Delete</t>
-        </is>
-      </c>
-      <c r="K11" s="4" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="L11" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> | Run: 2026-04-18 12:26 | Run: 2026-04-20 10:11 | Run: 2026-04-21 15:51</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t>TC-GEN-007</t>
-        </is>
-      </c>
-      <c r="B12" s="3" t="inlineStr">
-        <is>
-          <t>File &gt; 5MB → no client guard</t>
-        </is>
-      </c>
-      <c r="C12" s="3" t="inlineStr">
-        <is>
-          <t>CREATOR</t>
-        </is>
-      </c>
-      <c r="D12" s="3" t="inlineStr">
-        <is>
-          <t>PDF</t>
-        </is>
-      </c>
-      <c r="E12" s="3" t="inlineStr">
-        <is>
-          <t>data/sample_pdf_large.pdf</t>
-        </is>
-      </c>
-      <c r="F12" s="3" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="G12" s="3" t="inlineStr">
-        <is>
-          <t>Error: file too large</t>
-        </is>
-      </c>
-      <c r="H12" s="3" t="inlineStr">
-        <is>
-          <t>Sample large PDF not found at C:\quiz-trivia-tooltest\data\sample_pdf_large.pdf — place a file &gt;5MB there to run this TC</t>
-        </is>
-      </c>
-      <c r="I12" s="3" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="J12" s="3" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="K12" s="4" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="L12" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> | Run: 2026-04-18 12:26 | Run: 2026-04-20 10:12</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="5" t="inlineStr">
-        <is>
-          <t>TC-GEN-008</t>
-        </is>
-      </c>
-      <c r="B13" s="5" t="inlineStr">
-        <is>
-          <t>User role blocked from AI Generator</t>
-        </is>
-      </c>
-      <c r="C13" s="5" t="inlineStr">
-        <is>
-          <t>USER</t>
-        </is>
-      </c>
-      <c r="D13" s="5" t="inlineStr">
-        <is>
-          <t>Text</t>
-        </is>
-      </c>
-      <c r="E13" s="5" t="inlineStr">
-        <is>
-          <t>Tạo câu hỏi về lịch sử</t>
-        </is>
-      </c>
-      <c r="F13" s="5" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="G13" s="5" t="inlineStr">
-        <is>
-          <t>Access denied; AI Generator not visible</t>
-        </is>
-      </c>
-      <c r="H13" s="5" t="inlineStr">
-        <is>
-          <t>USER navigated to /creator/new → landed at: https://datn-quizapp.web.app/creator/new</t>
-        </is>
-      </c>
-      <c r="I13" s="5" t="inlineStr">
-        <is>
-          <t>No data saved (USER role blocked from creator route); Firestore role='creator'</t>
-        </is>
-      </c>
-      <c r="J13" s="5" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="K13" s="4" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="L13" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> | Run: 2026-04-18 12:26 | Run: 2026-04-20 10:13 | Run: 2026-04-21 15:54</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t>TC-GEN-009</t>
-        </is>
-      </c>
-      <c r="B14" s="3" t="inlineStr">
-        <is>
-          <t>Zero question types selected</t>
-        </is>
-      </c>
-      <c r="C14" s="3" t="inlineStr">
-        <is>
-          <t>CREATOR</t>
-        </is>
-      </c>
-      <c r="D14" s="3" t="inlineStr">
-        <is>
-          <t>Text</t>
-        </is>
-      </c>
-      <c r="E14" s="3" t="inlineStr">
-        <is>
-          <t>Tạo câu hỏi về khoa học</t>
-        </is>
-      </c>
-      <c r="F14" s="3" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="G14" s="3" t="inlineStr">
-        <is>
-          <t>Validation error; cannot submit</t>
-        </is>
-      </c>
-      <c r="H14" s="3" t="inlineStr">
-        <is>
-          <t>Toast on zero types: 'Đã tạo 5 câu hỏi!'; Preview opened: True</t>
-        </is>
-      </c>
-      <c r="I14" s="3" t="inlineStr">
-        <is>
-          <t>No DB write expected (should be blocked before API call)</t>
-        </is>
-      </c>
-      <c r="J14" s="3" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="K14" s="4" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="L14" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> | Run: 2026-04-18 12:26 | Run: 2026-04-20 10:15 | Run: 2026-04-21 16:17</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="25.5" customHeight="1">
-      <c r="A15" s="5" t="inlineStr">
-        <is>
-          <t>TC-GEN-010</t>
-        </is>
-      </c>
-      <c r="B15" s="5" t="inlineStr">
-        <is>
-          <t>Valid prompt → verify question schema</t>
-        </is>
-      </c>
-      <c r="C15" s="5" t="inlineStr">
-        <is>
-          <t>CREATOR</t>
-        </is>
-      </c>
-      <c r="D15" s="5" t="inlineStr">
-        <is>
-          <t>Text</t>
-        </is>
-      </c>
-      <c r="E15" s="5" t="inlineStr">
-        <is>
-          <t>Câu hỏi về công nghệ thông tin</t>
-        </is>
-      </c>
-      <c r="F15" s="5" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="G15" s="5" t="inlineStr">
-        <is>
-          <t>Questions shown with type, options, correct answer</t>
-        </is>
-      </c>
-      <c r="H15" s="5" t="inlineStr">
-        <is>
-          <t>Preview shows 5 question card(s). Toast: 'Đã tạo 5 câu hỏi!'</t>
-        </is>
-      </c>
-      <c r="I15" s="5" t="inlineStr">
-        <is>
-          <t>Found 5 question cards with text visible in preview</t>
-        </is>
-      </c>
-      <c r="J15" s="5" t="inlineStr">
-        <is>
-          <t>Delete</t>
-        </is>
-      </c>
-      <c r="K15" s="4" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="L15" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> | Run: 2026-04-18 12:27 | Run: 2026-04-20 10:16 | Run: 2026-04-21 16:24</t>
-        </is>
-      </c>
+      <c r="N15" s="16" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -1336,7 +1492,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:K17"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="36" customWidth="1" min="2" max="2"/>
@@ -1492,7 +1648,7 @@
         </is>
       </c>
     </row>
-    <row r="6">
+    <row r="6" ht="112.5" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
         <is>
           <t>TC-CB-002</t>
@@ -1551,7 +1707,7 @@
         </is>
       </c>
     </row>
-    <row r="7">
+    <row r="7" ht="37.5" customHeight="1">
       <c r="A7" s="5" t="inlineStr">
         <is>
           <t>TC-CB-003</t>
@@ -1847,7 +2003,7 @@
         </is>
       </c>
     </row>
-    <row r="12">
+    <row r="12" ht="162.5" customHeight="1">
       <c r="A12" s="3" t="inlineStr">
         <is>
           <t>TC-CB-011</t>
@@ -1967,7 +2123,7 @@
         </is>
       </c>
     </row>
-    <row r="14">
+    <row r="14" ht="162.5" customHeight="1">
       <c r="A14" s="3" t="inlineStr">
         <is>
           <t>TC-CB-031</t>
@@ -2141,7 +2297,7 @@
         </is>
       </c>
     </row>
-    <row r="17">
+    <row r="17" ht="37.5" customHeight="1">
       <c r="A17" s="5" t="inlineStr">
         <is>
           <t>TC-CB-024</t>

</xml_diff>